<commit_message>
More Work on Results Section!
</commit_message>
<xml_diff>
--- a/results/Segment_Shift_Tests.xlsx
+++ b/results/Segment_Shift_Tests.xlsx
@@ -660,7 +660,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>{'Early': 0.194184540287262, 'Late': 0.11819776965995085}</t>
+          <t>{'Early': 0.19418454028726198, 'Late': 0.11819776965995085}</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1630,7 +1630,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>{'1939': 0.05498663838448012, '1940': 0.1378478250744193, '1941': 0.21204424490976165, '1942': 0.11307231809803292, '1943': 0.06718596227188812, '1944': 0.025815108690527444, '1945': 0.02672727368210237}</t>
+          <t>{'1939': 0.05498663838448012, '1940': 0.1378478250744193, '1941': 0.21204424490976165, '1942': 0.11307231809803292, '1943': 0.0671859622718881, '1944': 0.025815108690527416, '1945': 0.02672727368210237}</t>
         </is>
       </c>
       <c r="J26" t="n">

</xml_diff>